<commit_message>
update index.html, Эталон_ПВЗ.xlsx, build_data.py to new versions
</commit_message>
<xml_diff>
--- a/Эталон_ПВЗ.xlsx
+++ b/Эталон_ПВЗ.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Справочник" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Заказы_по_неделям" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Объём_по_неделям" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочник" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Заказы_по_неделям" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объём_по_неделям" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -189,13 +189,10 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -214,20 +211,11 @@
     <xf numFmtId="9" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="4" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
@@ -279,9 +267,6 @@
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="4" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -568,861 +553,982 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="11" customWidth="1" style="23" min="1" max="1"/>
-    <col width="20" customWidth="1" style="23" min="2" max="2"/>
-    <col width="12" customWidth="1" style="23" min="3" max="3"/>
-    <col width="9" customWidth="1" style="23" min="4" max="5"/>
-    <col width="12" customWidth="1" style="23" min="6" max="6"/>
-    <col width="14" customWidth="1" style="23" min="7" max="7"/>
-    <col width="16" customWidth="1" style="23" min="8" max="8"/>
-    <col width="15" customWidth="1" style="23" min="9" max="9"/>
-    <col width="14" customWidth="1" style="23" min="10" max="10"/>
-    <col width="12" customWidth="1" style="23" min="11" max="11"/>
+    <col width="11" customWidth="1" style="19" min="1" max="1"/>
+    <col width="18" customWidth="1" style="19" min="2" max="2"/>
+    <col width="11" customWidth="1" style="19" min="3" max="3"/>
+    <col width="8" customWidth="1" style="19" min="4" max="4"/>
+    <col width="9" customWidth="1" style="19" min="5" max="5"/>
+    <col width="14" customWidth="1" style="19" min="6" max="6"/>
+    <col width="13" customWidth="1" style="19" min="7" max="7"/>
+    <col width="15" customWidth="1" style="19" min="8" max="8"/>
+    <col width="13" customWidth="1" style="19" min="9" max="9"/>
+    <col width="15" customWidth="1" style="19" min="10" max="10"/>
+    <col width="13" customWidth="1" style="19" min="11" max="11"/>
+    <col width="12" customWidth="1" style="19" min="12" max="12"/>
+    <col width="11" customWidth="1" style="19" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="24">
-      <c r="A1" s="25" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="20">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Эталон ПВЗ Uzum — справочник (источник правды для не-дневных параметров)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="24">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Синие — редактируемые входы. Заказы/выручка — на листах ниже, накапливаются из узум.xlsx через build_data.py.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="23.25" customHeight="1" s="24">
-      <c r="A4" s="27" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="20">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>Синие — редактируемые входы. OPEX = Аренда + ЗП (месячные, сум). Заказы/выручка — на листах ниже, накапливаются из узум.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="23.85" customHeight="1" s="20">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>Код</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="23" t="inlineStr">
         <is>
           <t>AKA</t>
         </is>
       </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="C4" s="23" t="inlineStr">
         <is>
           <t>Город</t>
         </is>
       </c>
-      <c r="D4" s="27" t="inlineStr">
+      <c r="D4" s="23" t="inlineStr">
         <is>
           <t>Сегмент</t>
         </is>
       </c>
-      <c r="E4" s="27" t="inlineStr">
+      <c r="E4" s="23" t="inlineStr">
         <is>
           <t>Комиссия</t>
         </is>
       </c>
-      <c r="F4" s="27" t="inlineStr">
-        <is>
-          <t>Опекс, $/мес</t>
-        </is>
-      </c>
-      <c r="G4" s="27" t="inlineStr">
+      <c r="F4" s="23" t="inlineStr">
+        <is>
+          <t>Аренда, сум/мес</t>
+        </is>
+      </c>
+      <c r="G4" s="23" t="inlineStr">
+        <is>
+          <t>ЗП, сум/мес</t>
+        </is>
+      </c>
+      <c r="H4" s="23" t="inlineStr">
         <is>
           <t>Затраты на УК, $/мес</t>
         </is>
       </c>
-      <c r="H4" s="27" t="inlineStr">
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>Разное, сум/мес</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr">
         <is>
           <t>Гарантия, сум/мес</t>
         </is>
       </c>
-      <c r="I4" s="27" t="inlineStr">
+      <c r="K4" s="23" t="inlineStr">
         <is>
           <t>Прогноз 1-го мес, зак/день</t>
         </is>
       </c>
-      <c r="J4" s="27" t="inlineStr">
+      <c r="L4" s="23" t="inlineStr">
         <is>
           <t>Яндекс-пик, зак/день</t>
         </is>
       </c>
-      <c r="K4" s="27" t="inlineStr">
+      <c r="M4" s="23" t="inlineStr">
         <is>
           <t>Старт</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="24">
-      <c r="A5" s="28" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="20">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>FRТАШ-290</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Буз-1</t>
         </is>
       </c>
-      <c r="C5" s="28" t="inlineStr">
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>Ташкент</t>
         </is>
       </c>
-      <c r="D5" s="29" t="n">
+      <c r="D5" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="30" t="n">
+      <c r="E5" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="F5" s="31" t="n">
-        <v>1327.87</v>
-      </c>
-      <c r="G5" s="32" t="n">
+      <c r="F5" s="27" t="n">
+        <v>6500000</v>
+      </c>
+      <c r="G5" s="27" t="n">
+        <v>9920000</v>
+      </c>
+      <c r="H5" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H5" s="32" t="n">
+      <c r="I5" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="27" t="n">
         <v>17400000</v>
       </c>
-      <c r="I5" s="29" t="n">
+      <c r="K5" s="25" t="n">
         <v>61</v>
       </c>
-      <c r="J5" s="29" t="n">
+      <c r="L5" s="25" t="n">
         <v>32</v>
       </c>
-      <c r="K5" s="33" t="inlineStr">
+      <c r="M5" s="28" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="24">
-      <c r="A6" s="28" t="inlineStr">
+    <row r="6" ht="15" customHeight="1" s="20">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>FRТАШ-291</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Бабур</t>
         </is>
       </c>
-      <c r="C6" s="28" t="inlineStr">
+      <c r="C6" s="24" t="inlineStr">
         <is>
           <t>Ташкент</t>
         </is>
       </c>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="30" t="n">
+      <c r="E6" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="F6" s="31" t="n">
-        <v>1524.59</v>
-      </c>
-      <c r="G6" s="32" t="n">
+      <c r="F6" s="27" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>9920000</v>
+      </c>
+      <c r="H6" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H6" s="32" t="n">
+      <c r="I6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="27" t="n">
         <v>17400000</v>
       </c>
-      <c r="I6" s="29" t="n">
+      <c r="K6" s="25" t="n">
         <v>39</v>
       </c>
-      <c r="J6" s="29" t="n">
+      <c r="L6" s="25" t="n">
         <v>43</v>
       </c>
-      <c r="K6" s="33" t="inlineStr">
+      <c r="M6" s="28" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="24">
-      <c r="A7" s="28" t="inlineStr">
+    <row r="7" ht="15" customHeight="1" s="20">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>FRТАШ-294</t>
         </is>
       </c>
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Шастри</t>
         </is>
       </c>
-      <c r="C7" s="28" t="inlineStr">
+      <c r="C7" s="24" t="inlineStr">
         <is>
           <t>Ташкент</t>
         </is>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="F7" s="31" t="n">
-        <v>1622.95</v>
-      </c>
-      <c r="G7" s="32" t="n">
+      <c r="F7" s="27" t="n">
+        <v>11909091</v>
+      </c>
+      <c r="G7" s="27" t="n">
+        <v>9920000</v>
+      </c>
+      <c r="H7" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H7" s="32" t="n">
+      <c r="I7" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="27" t="n">
         <v>17400000</v>
       </c>
-      <c r="I7" s="29" t="n">
+      <c r="K7" s="25" t="n">
         <v>38</v>
       </c>
-      <c r="J7" s="29" t="n">
+      <c r="L7" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="K7" s="33" t="inlineStr">
+      <c r="M7" s="28" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="24">
-      <c r="A8" s="28" t="inlineStr">
+    <row r="8" ht="15" customHeight="1" s="20">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>FRТАШ-292</t>
         </is>
       </c>
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>Спутник</t>
         </is>
       </c>
-      <c r="C8" s="28" t="inlineStr">
+      <c r="C8" s="24" t="inlineStr">
         <is>
           <t>Ташкент</t>
         </is>
       </c>
-      <c r="D8" s="29" t="n">
+      <c r="D8" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="30" t="n">
+      <c r="E8" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="F8" s="31" t="n">
-        <v>1131.15</v>
-      </c>
-      <c r="G8" s="32" t="n">
+      <c r="F8" s="27" t="n">
+        <v>3647160</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <v>9920000</v>
+      </c>
+      <c r="H8" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H8" s="32" t="n">
+      <c r="I8" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="27" t="n">
         <v>17400000</v>
       </c>
-      <c r="I8" s="29" t="n">
+      <c r="K8" s="25" t="n">
         <v>38</v>
       </c>
-      <c r="J8" s="29" t="n">
+      <c r="L8" s="25" t="n">
         <v>30</v>
       </c>
-      <c r="K8" s="33" t="inlineStr">
+      <c r="M8" s="28" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="24">
-      <c r="A9" s="28" t="inlineStr">
+    <row r="9" ht="15" customHeight="1" s="20">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>FRАЛМ-9</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>Алмалык Амир Т</t>
         </is>
       </c>
-      <c r="C9" s="28" t="inlineStr">
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>Алмалык</t>
         </is>
       </c>
-      <c r="D9" s="29" t="n">
+      <c r="D9" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="E9" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="F9" s="31" t="n">
-        <v>1032.79</v>
-      </c>
-      <c r="G9" s="32" t="n">
+      <c r="F9" s="27" t="n">
+        <v>4431000</v>
+      </c>
+      <c r="G9" s="27" t="n">
+        <v>8680000</v>
+      </c>
+      <c r="H9" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H9" s="32" t="n">
+      <c r="I9" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="27" t="n">
         <v>14000000</v>
       </c>
-      <c r="I9" s="29" t="n">
+      <c r="K9" s="25" t="n">
         <v>38</v>
       </c>
-      <c r="J9" s="29" t="n">
+      <c r="L9" s="25" t="n">
         <v>40</v>
       </c>
-      <c r="K9" s="33" t="inlineStr">
+      <c r="M9" s="28" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="24">
-      <c r="A10" s="28" t="inlineStr">
+    <row r="10" ht="15" customHeight="1" s="20">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>FRТАШ-289</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Афросиаб</t>
         </is>
       </c>
-      <c r="C10" s="28" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
         <is>
           <t>Ташкент</t>
         </is>
       </c>
-      <c r="D10" s="29" t="n">
+      <c r="D10" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="E10" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="F10" s="31" t="n">
-        <v>1524.59</v>
-      </c>
-      <c r="G10" s="32" t="n">
+      <c r="F10" s="27" t="n">
+        <v>10420455</v>
+      </c>
+      <c r="G10" s="27" t="n">
+        <v>9920000</v>
+      </c>
+      <c r="H10" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H10" s="32" t="n">
+      <c r="I10" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="27" t="n">
         <v>17400000</v>
       </c>
-      <c r="I10" s="29" t="n">
+      <c r="K10" s="25" t="n">
         <v>58</v>
       </c>
-      <c r="J10" s="29" t="n">
+      <c r="L10" s="25" t="n">
         <v>48</v>
       </c>
-      <c r="K10" s="33" t="inlineStr">
+      <c r="M10" s="28" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="24">
-      <c r="A11" s="28" t="inlineStr">
+    <row r="11" ht="15" customHeight="1" s="20">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>FRТАШ-293</t>
         </is>
       </c>
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Кургантепа</t>
         </is>
       </c>
-      <c r="C11" s="28" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
         <is>
           <t>Ташкент</t>
         </is>
       </c>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="30" t="n">
+      <c r="E11" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="F11" s="31" t="n">
-        <v>1327.87</v>
-      </c>
-      <c r="G11" s="32" t="n">
+      <c r="F11" s="27" t="n">
+        <v>7112000</v>
+      </c>
+      <c r="G11" s="27" t="n">
+        <v>9920000</v>
+      </c>
+      <c r="H11" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H11" s="32" t="n">
+      <c r="I11" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="27" t="n">
         <v>17400000</v>
       </c>
-      <c r="I11" s="29" t="n">
+      <c r="K11" s="25" t="n">
         <v>61</v>
       </c>
-      <c r="J11" s="29" t="n">
+      <c r="L11" s="25" t="n">
         <v>48</v>
       </c>
-      <c r="K11" s="33" t="inlineStr">
+      <c r="M11" s="28" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="24">
-      <c r="A12" s="28" t="inlineStr">
+    <row r="12" ht="15" customHeight="1" s="20">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>FRТАШ-319</t>
         </is>
       </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>Баку</t>
         </is>
       </c>
-      <c r="C12" s="28" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>Ташкент</t>
         </is>
       </c>
-      <c r="D12" s="29" t="n">
+      <c r="D12" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="30" t="n">
+      <c r="E12" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="F12" s="31" t="n">
-        <v>1229.51</v>
-      </c>
-      <c r="G12" s="32" t="n">
+      <c r="F12" s="27" t="n">
+        <v>5800000</v>
+      </c>
+      <c r="G12" s="27" t="n">
+        <v>9920000</v>
+      </c>
+      <c r="H12" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H12" s="32" t="n">
+      <c r="I12" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="27" t="n">
         <v>17400000</v>
       </c>
-      <c r="I12" s="29" t="n">
+      <c r="K12" s="25" t="n">
         <v>35</v>
       </c>
-      <c r="J12" s="29" t="n">
+      <c r="L12" s="25" t="n">
         <v>34</v>
       </c>
-      <c r="K12" s="33" t="inlineStr">
+      <c r="M12" s="28" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="24">
-      <c r="A13" s="28" t="inlineStr">
+    <row r="13" ht="15" customHeight="1" s="20">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>FRБХР-30</t>
         </is>
       </c>
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Бухара</t>
         </is>
       </c>
-      <c r="C13" s="28" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>Бухара</t>
         </is>
       </c>
-      <c r="D13" s="29" t="n">
+      <c r="D13" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="30" t="n">
+      <c r="E13" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="F13" s="31" t="n">
-        <v>1131.15</v>
-      </c>
-      <c r="G13" s="32" t="n">
+      <c r="F13" s="27" t="n">
+        <v>5818182</v>
+      </c>
+      <c r="G13" s="27" t="n">
+        <v>8680000</v>
+      </c>
+      <c r="H13" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H13" s="32" t="n">
+      <c r="I13" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="27" t="n">
         <v>14000000</v>
       </c>
-      <c r="I13" s="29" t="n">
+      <c r="K13" s="25" t="n">
         <v>31</v>
       </c>
-      <c r="J13" s="29" t="n">
+      <c r="L13" s="25" t="n">
         <v>25</v>
       </c>
-      <c r="K13" s="33" t="inlineStr">
+      <c r="M13" s="28" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="24">
-      <c r="A14" s="28" t="inlineStr">
+    <row r="14" ht="15" customHeight="1" s="20">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>FRГАЗ-4</t>
         </is>
       </c>
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>Газалкент</t>
         </is>
       </c>
-      <c r="C14" s="28" t="inlineStr">
+      <c r="C14" s="24" t="inlineStr">
         <is>
           <t>Газалкент</t>
         </is>
       </c>
-      <c r="D14" s="29" t="n">
+      <c r="D14" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="30" t="n">
+      <c r="E14" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="F14" s="31" t="n">
-        <v>934.4299999999999</v>
-      </c>
-      <c r="G14" s="32" t="n">
+      <c r="F14" s="27" t="n">
+        <v>2954545</v>
+      </c>
+      <c r="G14" s="27" t="n">
+        <v>7440000</v>
+      </c>
+      <c r="H14" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H14" s="32" t="n">
+      <c r="I14" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="27" t="n">
         <v>14000000</v>
       </c>
-      <c r="I14" s="29" t="n">
+      <c r="K14" s="25" t="n">
         <v>60</v>
       </c>
-      <c r="J14" s="29" t="n">
+      <c r="L14" s="25" t="n">
         <v>31</v>
       </c>
-      <c r="K14" s="33" t="inlineStr">
+      <c r="M14" s="28" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="24">
-      <c r="A15" s="28" t="inlineStr">
+    <row r="15" ht="15" customHeight="1" s="20">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>FRТАШ-308</t>
         </is>
       </c>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>Янгиюнусабад</t>
         </is>
       </c>
-      <c r="C15" s="28" t="inlineStr">
+      <c r="C15" s="24" t="inlineStr">
         <is>
           <t>Ташкент</t>
         </is>
       </c>
-      <c r="D15" s="29" t="n">
+      <c r="D15" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="30" t="n">
+      <c r="E15" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="F15" s="31" t="n">
-        <v>1327.87</v>
-      </c>
-      <c r="G15" s="32" t="n">
+      <c r="F15" s="27" t="n">
+        <v>7386364</v>
+      </c>
+      <c r="G15" s="27" t="n">
+        <v>9920000</v>
+      </c>
+      <c r="H15" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H15" s="32" t="n">
+      <c r="I15" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="27" t="n">
         <v>17400000</v>
       </c>
-      <c r="I15" s="29" t="n">
+      <c r="K15" s="25" t="n">
         <v>61</v>
       </c>
-      <c r="J15" s="29" t="n">
+      <c r="L15" s="25" t="n">
         <v>65</v>
       </c>
-      <c r="K15" s="33" t="inlineStr">
+      <c r="M15" s="28" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="24">
-      <c r="A16" s="28" t="inlineStr">
+    <row r="16" ht="15" customHeight="1" s="20">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>FRБУК-2</t>
         </is>
       </c>
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
         <is>
           <t>Бука</t>
         </is>
       </c>
-      <c r="C16" s="28" t="inlineStr">
+      <c r="C16" s="24" t="inlineStr">
         <is>
           <t>Бука</t>
         </is>
       </c>
-      <c r="D16" s="29" t="n">
+      <c r="D16" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="30" t="n">
+      <c r="E16" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="F16" s="31" t="n">
-        <v>934.4299999999999</v>
-      </c>
-      <c r="G16" s="32" t="n">
+      <c r="F16" s="27" t="n">
+        <v>2954545</v>
+      </c>
+      <c r="G16" s="27" t="n">
+        <v>7440000</v>
+      </c>
+      <c r="H16" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H16" s="32" t="n">
+      <c r="I16" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="27" t="n">
         <v>14000000</v>
       </c>
-      <c r="I16" s="29" t="n">
+      <c r="K16" s="25" t="n">
         <v>33</v>
       </c>
-      <c r="J16" s="29" t="n">
+      <c r="L16" s="25" t="n">
         <v>43</v>
       </c>
-      <c r="K16" s="33" t="inlineStr">
+      <c r="M16" s="28" t="inlineStr">
         <is>
           <t>2026-05-05</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1" s="24">
-      <c r="A17" s="28" t="inlineStr">
+    <row r="17" ht="15" customHeight="1" s="20">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>FRСМК-52</t>
         </is>
       </c>
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>Рудаки</t>
         </is>
       </c>
-      <c r="C17" s="28" t="inlineStr">
+      <c r="C17" s="24" t="inlineStr">
         <is>
           <t>Самарканд</t>
         </is>
       </c>
-      <c r="D17" s="29" t="n">
+      <c r="D17" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="30" t="n">
+      <c r="E17" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="F17" s="31" t="n">
-        <v>1278.69</v>
-      </c>
-      <c r="G17" s="32" t="n">
+      <c r="F17" s="27" t="n">
+        <v>7329545</v>
+      </c>
+      <c r="G17" s="27" t="n">
+        <v>8680000</v>
+      </c>
+      <c r="H17" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H17" s="32" t="n">
+      <c r="I17" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="27" t="n">
         <v>14000000</v>
       </c>
-      <c r="I17" s="29" t="n">
+      <c r="K17" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="J17" s="29" t="n">
+      <c r="L17" s="25" t="n">
         <v>41</v>
       </c>
-      <c r="K17" s="33" t="inlineStr">
+      <c r="M17" s="28" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="24">
-      <c r="A18" s="28" t="inlineStr">
+    <row r="18" ht="15" customHeight="1" s="20">
+      <c r="A18" s="24" t="inlineStr">
         <is>
           <t>FRАЛМ-10</t>
         </is>
       </c>
-      <c r="B18" s="28" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>Алмалык Мустакилик</t>
         </is>
       </c>
-      <c r="C18" s="28" t="inlineStr">
+      <c r="C18" s="24" t="inlineStr">
         <is>
           <t>Алмалык</t>
         </is>
       </c>
-      <c r="D18" s="29" t="n">
+      <c r="D18" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="30" t="n">
+      <c r="E18" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="F18" s="31" t="n">
-        <v>934.4299999999999</v>
-      </c>
-      <c r="G18" s="32" t="n">
+      <c r="F18" s="27" t="n">
+        <v>3409091</v>
+      </c>
+      <c r="G18" s="27" t="n">
+        <v>8680000</v>
+      </c>
+      <c r="H18" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H18" s="32" t="n">
+      <c r="I18" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="27" t="n">
         <v>14000000</v>
       </c>
-      <c r="I18" s="29" t="n">
+      <c r="K18" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="J18" s="29" t="n">
+      <c r="L18" s="25" t="n">
         <v>23</v>
       </c>
-      <c r="K18" s="33" t="inlineStr">
+      <c r="M18" s="28" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="24">
-      <c r="A19" s="28" t="inlineStr">
+    <row r="19" ht="15" customHeight="1" s="20">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>FRПСК-2</t>
         </is>
       </c>
-      <c r="B19" s="28" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Пскент</t>
         </is>
       </c>
-      <c r="C19" s="28" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>Пскент</t>
         </is>
       </c>
-      <c r="D19" s="29" t="n">
+      <c r="D19" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="30" t="n">
+      <c r="E19" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="F19" s="31" t="n">
-        <v>1032.79</v>
-      </c>
-      <c r="G19" s="32" t="n">
+      <c r="F19" s="27" t="n">
+        <v>4435000</v>
+      </c>
+      <c r="G19" s="27" t="n">
+        <v>7440000</v>
+      </c>
+      <c r="H19" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H19" s="32" t="n">
+      <c r="I19" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="27" t="n">
         <v>14000000</v>
       </c>
-      <c r="I19" s="29" t="n">
+      <c r="K19" s="25" t="n">
         <v>37</v>
       </c>
-      <c r="J19" s="29" t="n">
+      <c r="L19" s="25" t="n">
         <v>40</v>
       </c>
-      <c r="K19" s="33" t="inlineStr">
+      <c r="M19" s="28" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="24">
-      <c r="A20" s="28" t="inlineStr">
+    <row r="20" ht="15" customHeight="1" s="20">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>FRТАШ-307</t>
         </is>
       </c>
-      <c r="B20" s="28" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>Крестик</t>
         </is>
       </c>
-      <c r="C20" s="28" t="inlineStr">
+      <c r="C20" s="24" t="inlineStr">
         <is>
           <t>Ташкент</t>
         </is>
       </c>
-      <c r="D20" s="29" t="n">
+      <c r="D20" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="30" t="n">
+      <c r="E20" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="F20" s="31" t="n">
-        <v>1229.51</v>
-      </c>
-      <c r="G20" s="32" t="n">
+      <c r="F20" s="27" t="n">
+        <v>7216000</v>
+      </c>
+      <c r="G20" s="27" t="n">
+        <v>9920000</v>
+      </c>
+      <c r="H20" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H20" s="32" t="n">
+      <c r="I20" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="27" t="n">
         <v>17400000</v>
       </c>
-      <c r="I20" s="29" t="n">
+      <c r="K20" s="25" t="n">
         <v>60</v>
       </c>
-      <c r="J20" s="29" t="n">
+      <c r="L20" s="25" t="n">
         <v>68</v>
       </c>
-      <c r="K20" s="33" t="inlineStr">
+      <c r="M20" s="28" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="24">
-      <c r="A21" s="28" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="20">
+      <c r="A21" s="24" t="inlineStr">
         <is>
           <t>FRМРГ-8</t>
         </is>
       </c>
-      <c r="B21" s="28" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>Маргилан</t>
         </is>
       </c>
-      <c r="C21" s="28" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>Маргилан</t>
         </is>
       </c>
-      <c r="D21" s="29" t="n">
+      <c r="D21" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="E21" s="30" t="n">
+      <c r="E21" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="F21" s="31" t="n">
-        <v>934.4299999999999</v>
-      </c>
-      <c r="G21" s="32" t="n">
+      <c r="F21" s="27" t="n">
+        <v>2912000</v>
+      </c>
+      <c r="G21" s="27" t="n">
+        <v>8680000</v>
+      </c>
+      <c r="H21" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H21" s="32" t="n">
+      <c r="I21" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="27" t="n">
         <v>11400000</v>
       </c>
-      <c r="I21" s="29" t="n">
+      <c r="K21" s="25" t="n">
         <v>19</v>
       </c>
-      <c r="J21" s="29" t="n">
+      <c r="L21" s="25" t="n">
         <v>26</v>
       </c>
-      <c r="K21" s="33" t="inlineStr">
+      <c r="M21" s="28" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="24">
-      <c r="A22" s="28" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="20">
+      <c r="A22" s="24" t="inlineStr">
         <is>
           <t>FRСМК-53</t>
         </is>
       </c>
-      <c r="B22" s="28" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Андижанская</t>
         </is>
       </c>
-      <c r="C22" s="28" t="inlineStr">
+      <c r="C22" s="24" t="inlineStr">
         <is>
           <t>Самарканд</t>
         </is>
       </c>
-      <c r="D22" s="29" t="n">
+      <c r="D22" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="30" t="n">
+      <c r="E22" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="F22" s="31" t="n">
-        <v>1180.33</v>
-      </c>
-      <c r="G22" s="32" t="n">
+      <c r="F22" s="27" t="n">
+        <v>5864000</v>
+      </c>
+      <c r="G22" s="27" t="n">
+        <v>8680000</v>
+      </c>
+      <c r="H22" s="27" t="n">
         <v>320</v>
       </c>
-      <c r="H22" s="32" t="n">
+      <c r="I22" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="27" t="n">
         <v>14000000</v>
       </c>
-      <c r="I22" s="29" t="n">
+      <c r="K22" s="25" t="n">
         <v>24</v>
       </c>
-      <c r="J22" s="29" t="n">
+      <c r="L22" s="25" t="n">
         <v>29</v>
       </c>
-      <c r="K22" s="33" t="inlineStr">
+      <c r="M22" s="28" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -1444,29 +1550,29 @@
   <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="11" customWidth="1" style="23" min="1" max="1"/>
-    <col width="20" customWidth="1" style="23" min="2" max="2"/>
-    <col width="13" customWidth="1" style="23" min="3" max="6"/>
-    <col width="13" customWidth="1" style="24" min="4" max="4"/>
-    <col width="13" customWidth="1" style="24" min="5" max="5"/>
-    <col width="13" customWidth="1" style="24" min="6" max="6"/>
+    <col width="11" customWidth="1" style="19" min="1" max="1"/>
+    <col width="20" customWidth="1" style="19" min="2" max="2"/>
+    <col width="13" customWidth="1" style="19" min="3" max="6"/>
+    <col width="13" customWidth="1" style="20" min="4" max="4"/>
+    <col width="13" customWidth="1" style="20" min="5" max="5"/>
+    <col width="13" customWidth="1" style="20" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="24">
-      <c r="A1" s="34" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="20">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Средние заказы в день по неделям (накопительно)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="24">
-      <c r="A2" s="35" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="20">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>Накопительный архив: полные недели не меняются, последняя неполная — обновляется. Звёздочка = неполная неделя.</t>
         </is>
       </c>
     </row>
-    <row r="3" hidden="1" ht="15" customHeight="1" s="24">
+    <row r="3" hidden="1" ht="15" customHeight="1" s="20">
       <c r="C3" t="inlineStr">
         <is>
           <t>2026-05-11</t>
@@ -1488,510 +1594,510 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="24">
-      <c r="A4" s="36" t="inlineStr">
+    <row r="4" ht="15" customHeight="1" s="20">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>Код</t>
         </is>
       </c>
-      <c r="B4" s="36" t="inlineStr">
+      <c r="B4" s="31" t="inlineStr">
         <is>
           <t>AKA</t>
         </is>
       </c>
-      <c r="C4" s="36" t="inlineStr">
+      <c r="C4" s="31" t="inlineStr">
         <is>
           <t>11.05–17.05*</t>
         </is>
       </c>
-      <c r="D4" s="36" t="inlineStr">
+      <c r="D4" s="31" t="inlineStr">
         <is>
           <t>18.05–24.05</t>
         </is>
       </c>
-      <c r="E4" s="36" t="inlineStr">
+      <c r="E4" s="31" t="inlineStr">
         <is>
           <t>25.05–31.05</t>
         </is>
       </c>
-      <c r="F4" s="36" t="inlineStr">
+      <c r="F4" s="31" t="inlineStr">
         <is>
           <t>01.06–07.06*</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="24">
-      <c r="A5" s="37" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="20">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>Дней с данными</t>
         </is>
       </c>
-      <c r="B5" s="38" t="inlineStr"/>
-      <c r="C5" s="39" t="n">
+      <c r="B5" s="33" t="inlineStr"/>
+      <c r="C5" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="39" t="n">
+      <c r="D5" s="34" t="n">
         <v>7</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="E5" s="34" t="n">
         <v>7</v>
       </c>
-      <c r="F5" s="39" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="24">
-      <c r="A6" s="40" t="inlineStr">
+      <c r="F5" s="34" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="20">
+      <c r="A6" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-290</t>
         </is>
       </c>
-      <c r="B6" s="40" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>Буз-1</t>
         </is>
       </c>
-      <c r="C6" s="41" t="n">
+      <c r="C6" s="36" t="n">
         <v>30</v>
       </c>
-      <c r="D6" s="41" t="n">
+      <c r="D6" s="36" t="n">
         <v>37.86</v>
       </c>
-      <c r="E6" s="41" t="n">
+      <c r="E6" s="36" t="n">
         <v>39.57</v>
       </c>
-      <c r="F6" s="41" t="n">
-        <v>55.5</v>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="24">
-      <c r="A7" s="40" t="inlineStr">
+      <c r="F6" s="36" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="20">
+      <c r="A7" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-291</t>
         </is>
       </c>
-      <c r="B7" s="40" t="inlineStr">
+      <c r="B7" s="35" t="inlineStr">
         <is>
           <t>Бабур</t>
         </is>
       </c>
-      <c r="C7" s="41" t="n">
+      <c r="C7" s="36" t="n">
         <v>33.4</v>
       </c>
-      <c r="D7" s="41" t="n">
+      <c r="D7" s="36" t="n">
         <v>41.14</v>
       </c>
-      <c r="E7" s="41" t="n">
+      <c r="E7" s="36" t="n">
         <v>36.43</v>
       </c>
-      <c r="F7" s="41" t="n">
-        <v>52.5</v>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="24">
-      <c r="A8" s="40" t="inlineStr">
+      <c r="F7" s="36" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="20">
+      <c r="A8" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-292</t>
         </is>
       </c>
-      <c r="B8" s="40" t="inlineStr">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>Спутник</t>
         </is>
       </c>
-      <c r="C8" s="41" t="n">
+      <c r="C8" s="36" t="n">
         <v>18.6</v>
       </c>
-      <c r="D8" s="41" t="n">
+      <c r="D8" s="36" t="n">
         <v>21.57</v>
       </c>
-      <c r="E8" s="41" t="n">
+      <c r="E8" s="36" t="n">
         <v>26.14</v>
       </c>
-      <c r="F8" s="41" t="n">
-        <v>30.75</v>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="24">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="F8" s="36" t="n">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="20">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-294</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>Шастри</t>
+        </is>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>26.57</v>
+      </c>
+      <c r="E9" s="36" t="n">
+        <v>28.29</v>
+      </c>
+      <c r="F9" s="36" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="20">
+      <c r="A10" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-289</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>Афросиаб</t>
         </is>
       </c>
-      <c r="C9" s="41" t="n">
+      <c r="C10" s="36" t="n">
         <v>4.4</v>
       </c>
-      <c r="D9" s="41" t="n">
+      <c r="D10" s="36" t="n">
         <v>17.86</v>
       </c>
-      <c r="E9" s="41" t="n">
+      <c r="E10" s="36" t="n">
         <v>20.86</v>
       </c>
-      <c r="F9" s="41" t="n">
-        <v>23.25</v>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="24">
-      <c r="A10" s="40" t="inlineStr">
+      <c r="F10" s="36" t="n">
+        <v>20.5</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="20">
+      <c r="A11" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-293</t>
         </is>
       </c>
-      <c r="B10" s="40" t="inlineStr">
+      <c r="B11" s="35" t="inlineStr">
         <is>
           <t>Кургантепа</t>
         </is>
       </c>
-      <c r="C10" s="41" t="n">
+      <c r="C11" s="36" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="41" t="n">
+      <c r="D11" s="36" t="n">
         <v>13</v>
       </c>
-      <c r="E10" s="41" t="n">
+      <c r="E11" s="36" t="n">
         <v>17.71</v>
       </c>
-      <c r="F10" s="41" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="24">
-      <c r="A11" s="40" t="inlineStr">
-        <is>
-          <t>FRТАШ-294</t>
-        </is>
-      </c>
-      <c r="B11" s="40" t="inlineStr">
-        <is>
-          <t>Шастри</t>
-        </is>
-      </c>
-      <c r="C11" s="41" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="D11" s="41" t="n">
-        <v>26.57</v>
-      </c>
-      <c r="E11" s="41" t="n">
-        <v>28.29</v>
-      </c>
-      <c r="F11" s="41" t="n">
-        <v>22.75</v>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="24">
-      <c r="A12" s="40" t="inlineStr">
+      <c r="F11" s="36" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="20">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-319</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>Баку</t>
+        </is>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>19.43</v>
+      </c>
+      <c r="E12" s="36" t="n">
+        <v>15.71</v>
+      </c>
+      <c r="F12" s="36" t="n">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="20">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>FRАЛМ-9</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>Алмалык Амир Т</t>
+        </is>
+      </c>
+      <c r="C13" s="36" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="D13" s="36" t="n">
+        <v>16.57</v>
+      </c>
+      <c r="E13" s="36" t="n">
+        <v>20.86</v>
+      </c>
+      <c r="F13" s="36" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="20">
+      <c r="A14" s="35" t="inlineStr">
         <is>
           <t>FRБХР-30</t>
         </is>
       </c>
-      <c r="B12" s="40" t="inlineStr">
+      <c r="B14" s="35" t="inlineStr">
         <is>
           <t>Бухара</t>
         </is>
       </c>
-      <c r="C12" s="41" t="n">
+      <c r="C14" s="36" t="n">
         <v>13.8</v>
       </c>
-      <c r="D12" s="41" t="n">
+      <c r="D14" s="36" t="n">
         <v>21.71</v>
       </c>
-      <c r="E12" s="41" t="n">
+      <c r="E14" s="36" t="n">
         <v>15.43</v>
       </c>
-      <c r="F12" s="41" t="n">
-        <v>18.5</v>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="24">
-      <c r="A13" s="40" t="inlineStr">
-        <is>
-          <t>FRАЛМ-9</t>
-        </is>
-      </c>
-      <c r="B13" s="40" t="inlineStr">
-        <is>
-          <t>Алмалык Амир Т</t>
-        </is>
-      </c>
-      <c r="C13" s="41" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="D13" s="41" t="n">
-        <v>16.57</v>
-      </c>
-      <c r="E13" s="41" t="n">
-        <v>20.86</v>
-      </c>
-      <c r="F13" s="41" t="n">
-        <v>18.25</v>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="24">
-      <c r="A14" s="40" t="inlineStr">
+      <c r="F14" s="36" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="20">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>FRГАЗ-4</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>Газалкент</t>
+        </is>
+      </c>
+      <c r="C15" s="36" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="D15" s="36" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="E15" s="36" t="n">
+        <v>14.57</v>
+      </c>
+      <c r="F15" s="36" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="20">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>FRАЛМ-10</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>Алмалык Мустакилик</t>
+        </is>
+      </c>
+      <c r="C16" s="36" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="D16" s="36" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="E16" s="36" t="n">
+        <v>9.140000000000001</v>
+      </c>
+      <c r="F16" s="36" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="20">
+      <c r="A17" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-308</t>
         </is>
       </c>
-      <c r="B14" s="40" t="inlineStr">
+      <c r="B17" s="35" t="inlineStr">
         <is>
           <t>Янгиюнусабад</t>
         </is>
       </c>
-      <c r="C14" s="41" t="n">
+      <c r="C17" s="36" t="n">
         <v>10.8</v>
       </c>
-      <c r="D14" s="41" t="n">
+      <c r="D17" s="36" t="n">
         <v>13.57</v>
       </c>
-      <c r="E14" s="41" t="n">
+      <c r="E17" s="36" t="n">
         <v>12.57</v>
       </c>
-      <c r="F14" s="41" t="n">
-        <v>15.5</v>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="24">
-      <c r="A15" s="40" t="inlineStr">
-        <is>
-          <t>FRГАЗ-4</t>
-        </is>
-      </c>
-      <c r="B15" s="40" t="inlineStr">
-        <is>
-          <t>Газалкент</t>
-        </is>
-      </c>
-      <c r="C15" s="41" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="D15" s="41" t="n">
-        <v>13.29</v>
-      </c>
-      <c r="E15" s="41" t="n">
-        <v>14.57</v>
-      </c>
-      <c r="F15" s="41" t="n">
-        <v>14.25</v>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="24">
-      <c r="A16" s="40" t="inlineStr">
+      <c r="F17" s="36" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="20">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-307</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>Крестик</t>
+        </is>
+      </c>
+      <c r="C18" s="36" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D18" s="36" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="E18" s="36" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="F18" s="36" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="20">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>FRБУК-2</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>Бука</t>
+        </is>
+      </c>
+      <c r="C19" s="36" t="n">
+        <v>7</v>
+      </c>
+      <c r="D19" s="36" t="n">
+        <v>12.57</v>
+      </c>
+      <c r="E19" s="36" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="F19" s="36" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="20">
+      <c r="A20" s="35" t="inlineStr">
         <is>
           <t>FRСМК-52</t>
         </is>
       </c>
-      <c r="B16" s="40" t="inlineStr">
+      <c r="B20" s="35" t="inlineStr">
         <is>
           <t>Рудаки</t>
         </is>
       </c>
-      <c r="C16" s="41" t="n">
+      <c r="C20" s="36" t="n">
         <v>11</v>
       </c>
-      <c r="D16" s="41" t="n">
+      <c r="D20" s="36" t="n">
         <v>10.43</v>
       </c>
-      <c r="E16" s="41" t="n">
+      <c r="E20" s="36" t="n">
         <v>11.14</v>
       </c>
-      <c r="F16" s="41" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="24">
-      <c r="A17" s="40" t="inlineStr">
-        <is>
-          <t>FRТАШ-319</t>
-        </is>
-      </c>
-      <c r="B17" s="40" t="inlineStr">
-        <is>
-          <t>Баку</t>
-        </is>
-      </c>
-      <c r="C17" s="41" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="D17" s="41" t="n">
-        <v>19.43</v>
-      </c>
-      <c r="E17" s="41" t="n">
-        <v>15.71</v>
-      </c>
-      <c r="F17" s="41" t="n">
-        <v>13.75</v>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="24">
-      <c r="A18" s="40" t="inlineStr">
-        <is>
-          <t>FRАЛМ-10</t>
-        </is>
-      </c>
-      <c r="B18" s="40" t="inlineStr">
-        <is>
-          <t>Алмалык Мустакилик</t>
-        </is>
-      </c>
-      <c r="C18" s="41" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="D18" s="41" t="n">
-        <v>8.140000000000001</v>
-      </c>
-      <c r="E18" s="41" t="n">
-        <v>9.140000000000001</v>
-      </c>
-      <c r="F18" s="41" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="24">
-      <c r="A19" s="40" t="inlineStr">
-        <is>
-          <t>FRБУК-2</t>
-        </is>
-      </c>
-      <c r="B19" s="40" t="inlineStr">
-        <is>
-          <t>Бука</t>
-        </is>
-      </c>
-      <c r="C19" s="41" t="n">
+      <c r="F20" s="36" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="20">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>FRПСК-2</t>
+        </is>
+      </c>
+      <c r="B21" s="35" t="inlineStr">
+        <is>
+          <t>Пскент</t>
+        </is>
+      </c>
+      <c r="C21" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="36" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="E21" s="36" t="n">
         <v>7</v>
       </c>
-      <c r="D19" s="41" t="n">
-        <v>12.57</v>
-      </c>
-      <c r="E19" s="41" t="n">
-        <v>11.29</v>
-      </c>
-      <c r="F19" s="41" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="24">
-      <c r="A20" s="40" t="inlineStr">
-        <is>
-          <t>FRПСК-2</t>
-        </is>
-      </c>
-      <c r="B20" s="40" t="inlineStr">
-        <is>
-          <t>Пскент</t>
-        </is>
-      </c>
-      <c r="C20" s="41" t="n">
+      <c r="F21" s="36" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="20">
+      <c r="A22" s="35" t="inlineStr">
+        <is>
+          <t>FRМРГ-8</t>
+        </is>
+      </c>
+      <c r="B22" s="35" t="inlineStr">
+        <is>
+          <t>Маргилан</t>
+        </is>
+      </c>
+      <c r="C22" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="D20" s="41" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="E20" s="41" t="n">
-        <v>7</v>
-      </c>
-      <c r="F20" s="41" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="24">
-      <c r="A21" s="40" t="inlineStr">
-        <is>
-          <t>FRТАШ-307</t>
-        </is>
-      </c>
-      <c r="B21" s="40" t="inlineStr">
-        <is>
-          <t>Крестик</t>
-        </is>
-      </c>
-      <c r="C21" s="41" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D21" s="41" t="n">
-        <v>5.14</v>
-      </c>
-      <c r="E21" s="41" t="n">
-        <v>5.29</v>
-      </c>
-      <c r="F21" s="41" t="n">
+      <c r="D22" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="36" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="F22" s="36" t="n">
         <v>8.5</v>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="24">
-      <c r="A22" s="40" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="20">
+      <c r="A23" s="35" t="inlineStr">
         <is>
           <t>FRСМК-53</t>
         </is>
       </c>
-      <c r="B22" s="40" t="inlineStr">
+      <c r="B23" s="35" t="inlineStr">
         <is>
           <t>Андижанская</t>
         </is>
       </c>
-      <c r="C22" s="41" t="n">
+      <c r="C23" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="41" t="n">
+      <c r="D23" s="36" t="n">
         <v>0.14</v>
       </c>
-      <c r="E22" s="41" t="n">
+      <c r="E23" s="36" t="n">
         <v>2.86</v>
       </c>
-      <c r="F22" s="41" t="n">
-        <v>6.75</v>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="24">
-      <c r="A23" s="40" t="inlineStr">
-        <is>
-          <t>FRМРГ-8</t>
-        </is>
-      </c>
-      <c r="B23" s="40" t="inlineStr">
-        <is>
-          <t>Маргилан</t>
-        </is>
-      </c>
-      <c r="C23" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="41" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="41" t="n">
-        <v>3.86</v>
-      </c>
-      <c r="F23" s="41" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="24">
-      <c r="A24" s="42" t="inlineStr">
+      <c r="F23" s="36" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="20">
+      <c r="A24" s="37" t="inlineStr">
         <is>
           <t>В среднем на ПВЗ</t>
         </is>
       </c>
-      <c r="B24" s="43" t="inlineStr"/>
-      <c r="C24" s="44">
+      <c r="B24" s="38" t="inlineStr"/>
+      <c r="C24" s="39">
         <f>AVERAGE(C6:C23)</f>
         <v/>
       </c>
-      <c r="D24" s="44">
+      <c r="D24" s="39">
         <f>AVERAGE(D6:D23)</f>
         <v/>
       </c>
-      <c r="E24" s="44">
+      <c r="E24" s="39">
         <f>AVERAGE(E6:E23)</f>
         <v/>
       </c>
-      <c r="F24" s="44">
+      <c r="F24" s="39">
         <f>AVERAGE(F6:F23)</f>
         <v/>
       </c>
@@ -2012,29 +2118,29 @@
   <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="11" customWidth="1" style="23" min="1" max="1"/>
-    <col width="20" customWidth="1" style="23" min="2" max="2"/>
-    <col width="13" customWidth="1" style="23" min="3" max="6"/>
-    <col width="13" customWidth="1" style="24" min="4" max="4"/>
-    <col width="13" customWidth="1" style="24" min="5" max="5"/>
-    <col width="13" customWidth="1" style="24" min="6" max="6"/>
+    <col width="11" customWidth="1" style="19" min="1" max="1"/>
+    <col width="20" customWidth="1" style="19" min="2" max="2"/>
+    <col width="13" customWidth="1" style="19" min="3" max="6"/>
+    <col width="13" customWidth="1" style="20" min="4" max="4"/>
+    <col width="13" customWidth="1" style="20" min="5" max="5"/>
+    <col width="13" customWidth="1" style="20" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="24">
-      <c r="A1" s="34" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="20">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Сумма выручки (объём) по неделям, сум (накопительно)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="24">
-      <c r="A2" s="35" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="20">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>Накопительный архив: полные недели не меняются, последняя неполная — обновляется. Звёздочка = неполная неделя.</t>
         </is>
       </c>
     </row>
-    <row r="3" hidden="1" ht="15" customHeight="1" s="24">
+    <row r="3" hidden="1" ht="15" customHeight="1" s="20">
       <c r="C3" t="inlineStr">
         <is>
           <t>2026-05-11</t>
@@ -2056,510 +2162,510 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="24">
-      <c r="A4" s="36" t="inlineStr">
+    <row r="4" ht="15" customHeight="1" s="20">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>Код</t>
         </is>
       </c>
-      <c r="B4" s="36" t="inlineStr">
+      <c r="B4" s="31" t="inlineStr">
         <is>
           <t>AKA</t>
         </is>
       </c>
-      <c r="C4" s="36" t="inlineStr">
+      <c r="C4" s="31" t="inlineStr">
         <is>
           <t>11.05–17.05*</t>
         </is>
       </c>
-      <c r="D4" s="36" t="inlineStr">
+      <c r="D4" s="31" t="inlineStr">
         <is>
           <t>18.05–24.05</t>
         </is>
       </c>
-      <c r="E4" s="36" t="inlineStr">
+      <c r="E4" s="31" t="inlineStr">
         <is>
           <t>25.05–31.05</t>
         </is>
       </c>
-      <c r="F4" s="36" t="inlineStr">
+      <c r="F4" s="31" t="inlineStr">
         <is>
           <t>01.06–07.06*</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="24">
-      <c r="A5" s="37" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="20">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>Дней с данными</t>
         </is>
       </c>
-      <c r="B5" s="38" t="inlineStr"/>
-      <c r="C5" s="39" t="n">
+      <c r="B5" s="33" t="inlineStr"/>
+      <c r="C5" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="39" t="n">
+      <c r="D5" s="34" t="n">
         <v>7</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="E5" s="34" t="n">
         <v>7</v>
       </c>
-      <c r="F5" s="39" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="24">
-      <c r="A6" s="40" t="inlineStr">
+      <c r="F5" s="34" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="20">
+      <c r="A6" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-290</t>
         </is>
       </c>
-      <c r="B6" s="40" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>Буз-1</t>
         </is>
       </c>
-      <c r="C6" s="45" t="n">
+      <c r="C6" s="40" t="n">
         <v>26572309</v>
       </c>
-      <c r="D6" s="45" t="n">
+      <c r="D6" s="40" t="n">
         <v>54415488</v>
       </c>
-      <c r="E6" s="45" t="n">
+      <c r="E6" s="40" t="n">
         <v>46859038</v>
       </c>
-      <c r="F6" s="45" t="n">
-        <v>31785581</v>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="24">
-      <c r="A7" s="40" t="inlineStr">
+      <c r="F6" s="40" t="n">
+        <v>22088856</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="20">
+      <c r="A7" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-291</t>
         </is>
       </c>
-      <c r="B7" s="40" t="inlineStr">
+      <c r="B7" s="35" t="inlineStr">
         <is>
           <t>Бабур</t>
         </is>
       </c>
-      <c r="C7" s="45" t="n">
+      <c r="C7" s="40" t="n">
         <v>25945431</v>
       </c>
-      <c r="D7" s="45" t="n">
+      <c r="D7" s="40" t="n">
         <v>37459210</v>
       </c>
-      <c r="E7" s="45" t="n">
+      <c r="E7" s="40" t="n">
         <v>48992678</v>
       </c>
-      <c r="F7" s="45" t="n">
-        <v>35581023</v>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="24">
-      <c r="A8" s="40" t="inlineStr">
+      <c r="F7" s="40" t="n">
+        <v>7192321</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="20">
+      <c r="A8" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-292</t>
         </is>
       </c>
-      <c r="B8" s="40" t="inlineStr">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>Спутник</t>
         </is>
       </c>
-      <c r="C8" s="45" t="n">
+      <c r="C8" s="40" t="n">
         <v>14023998</v>
       </c>
-      <c r="D8" s="45" t="n">
+      <c r="D8" s="40" t="n">
         <v>23623555</v>
       </c>
-      <c r="E8" s="45" t="n">
+      <c r="E8" s="40" t="n">
         <v>37049808</v>
       </c>
-      <c r="F8" s="45" t="n">
-        <v>25462608</v>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="24">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="F8" s="40" t="n">
+        <v>15343237</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="20">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-294</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>Шастри</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>11787061</v>
+      </c>
+      <c r="D9" s="40" t="n">
+        <v>33489630</v>
+      </c>
+      <c r="E9" s="40" t="n">
+        <v>34406847</v>
+      </c>
+      <c r="F9" s="40" t="n">
+        <v>4614543</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="20">
+      <c r="A10" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-289</t>
         </is>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>Афросиаб</t>
         </is>
       </c>
-      <c r="C9" s="45" t="n">
+      <c r="C10" s="40" t="n">
         <v>3579870</v>
       </c>
-      <c r="D9" s="45" t="n">
+      <c r="D10" s="40" t="n">
         <v>26016508</v>
       </c>
-      <c r="E9" s="45" t="n">
+      <c r="E10" s="40" t="n">
         <v>28967720</v>
       </c>
-      <c r="F9" s="45" t="n">
-        <v>21236946</v>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="24">
-      <c r="A10" s="40" t="inlineStr">
+      <c r="F10" s="40" t="n">
+        <v>8017702</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="20">
+      <c r="A11" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-293</t>
         </is>
       </c>
-      <c r="B10" s="40" t="inlineStr">
+      <c r="B11" s="35" t="inlineStr">
         <is>
           <t>Кургантепа</t>
         </is>
       </c>
-      <c r="C10" s="45" t="n">
+      <c r="C11" s="40" t="n">
         <v>9063650</v>
       </c>
-      <c r="D10" s="45" t="n">
+      <c r="D11" s="40" t="n">
         <v>19435779</v>
       </c>
-      <c r="E10" s="45" t="n">
+      <c r="E11" s="40" t="n">
         <v>20382320</v>
       </c>
-      <c r="F10" s="45" t="n">
-        <v>10697485</v>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="24">
-      <c r="A11" s="40" t="inlineStr">
-        <is>
-          <t>FRТАШ-294</t>
-        </is>
-      </c>
-      <c r="B11" s="40" t="inlineStr">
-        <is>
-          <t>Шастри</t>
-        </is>
-      </c>
-      <c r="C11" s="45" t="n">
-        <v>11787061</v>
-      </c>
-      <c r="D11" s="45" t="n">
-        <v>33489630</v>
-      </c>
-      <c r="E11" s="45" t="n">
-        <v>34406847</v>
-      </c>
-      <c r="F11" s="45" t="n">
-        <v>15532201</v>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="24">
-      <c r="A12" s="40" t="inlineStr">
+      <c r="F11" s="40" t="n">
+        <v>3952124</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="20">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-319</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>Баку</t>
+        </is>
+      </c>
+      <c r="C12" s="40" t="n">
+        <v>11237754</v>
+      </c>
+      <c r="D12" s="40" t="n">
+        <v>29303296</v>
+      </c>
+      <c r="E12" s="40" t="n">
+        <v>17092421</v>
+      </c>
+      <c r="F12" s="40" t="n">
+        <v>7508366</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="20">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>FRАЛМ-9</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>Алмалык Амир Т</t>
+        </is>
+      </c>
+      <c r="C13" s="40" t="n">
+        <v>13421812</v>
+      </c>
+      <c r="D13" s="40" t="n">
+        <v>19296100</v>
+      </c>
+      <c r="E13" s="40" t="n">
+        <v>32898025</v>
+      </c>
+      <c r="F13" s="40" t="n">
+        <v>6157955</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="20">
+      <c r="A14" s="35" t="inlineStr">
         <is>
           <t>FRБХР-30</t>
         </is>
       </c>
-      <c r="B12" s="40" t="inlineStr">
+      <c r="B14" s="35" t="inlineStr">
         <is>
           <t>Бухара</t>
         </is>
       </c>
-      <c r="C12" s="45" t="n">
+      <c r="C14" s="40" t="n">
         <v>10462042</v>
       </c>
-      <c r="D12" s="45" t="n">
+      <c r="D14" s="40" t="n">
         <v>24242808</v>
       </c>
-      <c r="E12" s="45" t="n">
+      <c r="E14" s="40" t="n">
         <v>20176647</v>
       </c>
-      <c r="F12" s="45" t="n">
-        <v>8986966</v>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="24">
-      <c r="A13" s="40" t="inlineStr">
-        <is>
-          <t>FRАЛМ-9</t>
-        </is>
-      </c>
-      <c r="B13" s="40" t="inlineStr">
-        <is>
-          <t>Алмалык Амир Т</t>
-        </is>
-      </c>
-      <c r="C13" s="45" t="n">
-        <v>13421812</v>
-      </c>
-      <c r="D13" s="45" t="n">
-        <v>19296100</v>
-      </c>
-      <c r="E13" s="45" t="n">
-        <v>32898025</v>
-      </c>
-      <c r="F13" s="45" t="n">
-        <v>12540076</v>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="24">
-      <c r="A14" s="40" t="inlineStr">
+      <c r="F14" s="40" t="n">
+        <v>3643570</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="20">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>FRГАЗ-4</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>Газалкент</t>
+        </is>
+      </c>
+      <c r="C15" s="40" t="n">
+        <v>6139086</v>
+      </c>
+      <c r="D15" s="40" t="n">
+        <v>14744333</v>
+      </c>
+      <c r="E15" s="40" t="n">
+        <v>18390296</v>
+      </c>
+      <c r="F15" s="40" t="n">
+        <v>6589707</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="20">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>FRАЛМ-10</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>Алмалык Мустакилик</t>
+        </is>
+      </c>
+      <c r="C16" s="40" t="n">
+        <v>6011315</v>
+      </c>
+      <c r="D16" s="40" t="n">
+        <v>10213590</v>
+      </c>
+      <c r="E16" s="40" t="n">
+        <v>10032796</v>
+      </c>
+      <c r="F16" s="40" t="n">
+        <v>5098524</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="20">
+      <c r="A17" s="35" t="inlineStr">
         <is>
           <t>FRТАШ-308</t>
         </is>
       </c>
-      <c r="B14" s="40" t="inlineStr">
+      <c r="B17" s="35" t="inlineStr">
         <is>
           <t>Янгиюнусабад</t>
         </is>
       </c>
-      <c r="C14" s="45" t="n">
+      <c r="C17" s="40" t="n">
         <v>7434617</v>
       </c>
-      <c r="D14" s="45" t="n">
+      <c r="D17" s="40" t="n">
         <v>11541808</v>
       </c>
-      <c r="E14" s="45" t="n">
+      <c r="E17" s="40" t="n">
         <v>11589026</v>
       </c>
-      <c r="F14" s="45" t="n">
-        <v>13830368</v>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="24">
-      <c r="A15" s="40" t="inlineStr">
-        <is>
-          <t>FRГАЗ-4</t>
-        </is>
-      </c>
-      <c r="B15" s="40" t="inlineStr">
-        <is>
-          <t>Газалкент</t>
-        </is>
-      </c>
-      <c r="C15" s="45" t="n">
-        <v>6139086</v>
-      </c>
-      <c r="D15" s="45" t="n">
-        <v>14744333</v>
-      </c>
-      <c r="E15" s="45" t="n">
-        <v>18390296</v>
-      </c>
-      <c r="F15" s="45" t="n">
-        <v>11768949</v>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="24">
-      <c r="A16" s="40" t="inlineStr">
+      <c r="F17" s="40" t="n">
+        <v>3737498</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="20">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-307</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>Крестик</t>
+        </is>
+      </c>
+      <c r="C18" s="40" t="n">
+        <v>2876909</v>
+      </c>
+      <c r="D18" s="40" t="n">
+        <v>6793378</v>
+      </c>
+      <c r="E18" s="40" t="n">
+        <v>3855907</v>
+      </c>
+      <c r="F18" s="40" t="n">
+        <v>2500720</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="20">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>FRБУК-2</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>Бука</t>
+        </is>
+      </c>
+      <c r="C19" s="40" t="n">
+        <v>6458596</v>
+      </c>
+      <c r="D19" s="40" t="n">
+        <v>16321651</v>
+      </c>
+      <c r="E19" s="40" t="n">
+        <v>12911381</v>
+      </c>
+      <c r="F19" s="40" t="n">
+        <v>2821800</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="20">
+      <c r="A20" s="35" t="inlineStr">
         <is>
           <t>FRСМК-52</t>
         </is>
       </c>
-      <c r="B16" s="40" t="inlineStr">
+      <c r="B20" s="35" t="inlineStr">
         <is>
           <t>Рудаки</t>
         </is>
       </c>
-      <c r="C16" s="45" t="n">
+      <c r="C20" s="40" t="n">
         <v>6460094</v>
       </c>
-      <c r="D16" s="45" t="n">
+      <c r="D20" s="40" t="n">
         <v>14908071</v>
       </c>
-      <c r="E16" s="45" t="n">
+      <c r="E20" s="40" t="n">
         <v>20904887</v>
       </c>
-      <c r="F16" s="45" t="n">
-        <v>7784127</v>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="24">
-      <c r="A17" s="40" t="inlineStr">
-        <is>
-          <t>FRТАШ-319</t>
-        </is>
-      </c>
-      <c r="B17" s="40" t="inlineStr">
-        <is>
-          <t>Баку</t>
-        </is>
-      </c>
-      <c r="C17" s="45" t="n">
-        <v>11237754</v>
-      </c>
-      <c r="D17" s="45" t="n">
-        <v>29303296</v>
-      </c>
-      <c r="E17" s="45" t="n">
-        <v>17092421</v>
-      </c>
-      <c r="F17" s="45" t="n">
-        <v>10612356</v>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="24">
-      <c r="A18" s="40" t="inlineStr">
-        <is>
-          <t>FRАЛМ-10</t>
-        </is>
-      </c>
-      <c r="B18" s="40" t="inlineStr">
-        <is>
-          <t>Алмалык Мустакилик</t>
-        </is>
-      </c>
-      <c r="C18" s="45" t="n">
-        <v>6011315</v>
-      </c>
-      <c r="D18" s="45" t="n">
-        <v>10213590</v>
-      </c>
-      <c r="E18" s="45" t="n">
-        <v>10032796</v>
-      </c>
-      <c r="F18" s="45" t="n">
-        <v>12192687</v>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="24">
-      <c r="A19" s="40" t="inlineStr">
-        <is>
-          <t>FRБУК-2</t>
-        </is>
-      </c>
-      <c r="B19" s="40" t="inlineStr">
-        <is>
-          <t>Бука</t>
-        </is>
-      </c>
-      <c r="C19" s="45" t="n">
-        <v>6458596</v>
-      </c>
-      <c r="D19" s="45" t="n">
-        <v>16321651</v>
-      </c>
-      <c r="E19" s="45" t="n">
-        <v>12911381</v>
-      </c>
-      <c r="F19" s="45" t="n">
-        <v>8820297</v>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="24">
-      <c r="A20" s="40" t="inlineStr">
+      <c r="F20" s="40" t="n">
+        <v>3500535</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="20">
+      <c r="A21" s="35" t="inlineStr">
         <is>
           <t>FRПСК-2</t>
         </is>
       </c>
-      <c r="B20" s="40" t="inlineStr">
+      <c r="B21" s="35" t="inlineStr">
         <is>
           <t>Пскент</t>
         </is>
       </c>
-      <c r="C20" s="45" t="n">
+      <c r="C21" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="D20" s="45" t="n">
+      <c r="D21" s="40" t="n">
         <v>1357510</v>
       </c>
-      <c r="E20" s="45" t="n">
+      <c r="E21" s="40" t="n">
         <v>9736256</v>
       </c>
-      <c r="F20" s="45" t="n">
-        <v>5155323</v>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="24">
-      <c r="A21" s="40" t="inlineStr">
-        <is>
-          <t>FRТАШ-307</t>
-        </is>
-      </c>
-      <c r="B21" s="40" t="inlineStr">
-        <is>
-          <t>Крестик</t>
-        </is>
-      </c>
-      <c r="C21" s="45" t="n">
-        <v>2876909</v>
-      </c>
-      <c r="D21" s="45" t="n">
-        <v>6793378</v>
-      </c>
-      <c r="E21" s="45" t="n">
-        <v>3855907</v>
-      </c>
-      <c r="F21" s="45" t="n">
-        <v>4450940</v>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="24">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="F21" s="40" t="n">
+        <v>2131223</v>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="20">
+      <c r="A22" s="35" t="inlineStr">
+        <is>
+          <t>FRМРГ-8</t>
+        </is>
+      </c>
+      <c r="B22" s="35" t="inlineStr">
+        <is>
+          <t>Маргилан</t>
+        </is>
+      </c>
+      <c r="C22" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="40" t="n">
+        <v>1377990</v>
+      </c>
+      <c r="E22" s="40" t="n">
+        <v>3465270</v>
+      </c>
+      <c r="F22" s="40" t="n">
+        <v>3033290</v>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="20">
+      <c r="A23" s="35" t="inlineStr">
         <is>
           <t>FRСМК-53</t>
         </is>
       </c>
-      <c r="B22" s="40" t="inlineStr">
+      <c r="B23" s="35" t="inlineStr">
         <is>
           <t>Андижанская</t>
         </is>
       </c>
-      <c r="C22" s="45" t="n">
+      <c r="C23" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="45" t="n">
+      <c r="D23" s="40" t="n">
         <v>363900</v>
       </c>
-      <c r="E22" s="45" t="n">
+      <c r="E23" s="40" t="n">
         <v>3477490</v>
       </c>
-      <c r="F22" s="45" t="n">
-        <v>3735640</v>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="24">
-      <c r="A23" s="40" t="inlineStr">
-        <is>
-          <t>FRМРГ-8</t>
-        </is>
-      </c>
-      <c r="B23" s="40" t="inlineStr">
-        <is>
-          <t>Маргилан</t>
-        </is>
-      </c>
-      <c r="C23" s="45" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="45" t="n">
-        <v>1377990</v>
-      </c>
-      <c r="E23" s="45" t="n">
-        <v>3465270</v>
-      </c>
-      <c r="F23" s="45" t="n">
-        <v>3454610</v>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="24">
-      <c r="A24" s="42" t="inlineStr">
+      <c r="F23" s="40" t="n">
+        <v>2293470</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="20">
+      <c r="A24" s="37" t="inlineStr">
         <is>
           <t>В среднем на ПВЗ</t>
         </is>
       </c>
-      <c r="B24" s="43" t="inlineStr"/>
-      <c r="C24" s="46">
+      <c r="B24" s="38" t="inlineStr"/>
+      <c r="C24" s="41">
         <f>AVERAGE(C6:C23)</f>
         <v/>
       </c>
-      <c r="D24" s="46">
+      <c r="D24" s="41">
         <f>AVERAGE(D6:D23)</f>
         <v/>
       </c>
-      <c r="E24" s="46">
+      <c r="E24" s="41">
         <f>AVERAGE(E6:E23)</f>
         <v/>
       </c>
-      <c r="F24" s="46">
+      <c r="F24" s="41">
         <f>AVERAGE(F6:F23)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
satori: monthly fact pipeline — build_satori.py + Сатори_факт sheet + FACT in dashboard (fact P&L replaces model by default), /satori command, docs
</commit_message>
<xml_diff>
--- a/Эталон_ПВЗ.xlsx
+++ b/Эталон_ПВЗ.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочник" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Заказы_по_неделям" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объём_по_неделям" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Справочник" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Заказы_по_неделям" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Объём_по_неделям" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Сатори_факт" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -1573,22 +1574,22 @@
       </c>
     </row>
     <row r="3" hidden="1" ht="15" customHeight="1" s="20">
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
@@ -2141,22 +2142,22 @@
       </c>
     </row>
     <row r="3" hidden="1" ht="15" customHeight="1" s="20">
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
@@ -2675,4 +2676,354 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" style="20" min="1" max="1"/>
+    <col width="22" customWidth="1" style="20" min="2" max="2"/>
+    <col width="15" customWidth="1" style="20" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>Факт по отчётам «Сатори» (агентское вознаграждение Uzum), сум — накопительно по месяцам</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Доход ПВЗ = фикс. вознаграждение (гарантия, прорейчено) + п.1.8 + компенсация п.5.2.1. Закрытые месяцы не переписываются.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" hidden="1" s="20">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Код</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>AKA</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>май 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>Дней в месяце</t>
+        </is>
+      </c>
+      <c r="B5" s="33" t="inlineStr"/>
+      <c r="C5" s="34" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-290</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Буз-1</t>
+        </is>
+      </c>
+      <c r="C6" s="40" t="n">
+        <v>14619948</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-291</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Бабур</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>14598348</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-294</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>Шастри</t>
+        </is>
+      </c>
+      <c r="C8" s="40" t="n">
+        <v>23504800</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-292</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>Спутник</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>14593548</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>FRАЛМ-9</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>Алмалык Амир Т</t>
+        </is>
+      </c>
+      <c r="C10" s="40" t="n">
+        <v>11291523</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-289</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>Афросиаб</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="n">
+        <v>10117626</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-293</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>Кургантепа</t>
+        </is>
+      </c>
+      <c r="C12" s="40" t="n">
+        <v>11234206</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-319</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>Баку</t>
+        </is>
+      </c>
+      <c r="C13" s="40" t="n">
+        <v>14598348</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>FRБХР-30</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>Бухара</t>
+        </is>
+      </c>
+      <c r="C14" s="40" t="n">
+        <v>14003600</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>FRГАЗ-4</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>Газалкент</t>
+        </is>
+      </c>
+      <c r="C15" s="40" t="n">
+        <v>14001200</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-308</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>Янгиюнусабад</t>
+        </is>
+      </c>
+      <c r="C16" s="40" t="n">
+        <v>17401200</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>FRБУК-2</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>Бука</t>
+        </is>
+      </c>
+      <c r="C17" s="40" t="n">
+        <v>12193548</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>FRСМК-52</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>Рудаки</t>
+        </is>
+      </c>
+      <c r="C18" s="40" t="n">
+        <v>12645161</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>FRАЛМ-10</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>Алмалык Мустакилик</t>
+        </is>
+      </c>
+      <c r="C19" s="40" t="n">
+        <v>11744335</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>FRПСК-2</t>
+        </is>
+      </c>
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>Пскент</t>
+        </is>
+      </c>
+      <c r="C20" s="40" t="n">
+        <v>5422955</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>FRТАШ-307</t>
+        </is>
+      </c>
+      <c r="B21" s="35" t="inlineStr">
+        <is>
+          <t>Крестик</t>
+        </is>
+      </c>
+      <c r="C21" s="40" t="n">
+        <v>23501200</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="35" t="inlineStr">
+        <is>
+          <t>FRМРГ-8</t>
+        </is>
+      </c>
+      <c r="B22" s="35" t="inlineStr">
+        <is>
+          <t>Маргилан</t>
+        </is>
+      </c>
+      <c r="C22" s="40" t="n">
+        <v>5148387</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="35" t="inlineStr">
+        <is>
+          <t>FRСМК-53</t>
+        </is>
+      </c>
+      <c r="B23" s="35" t="inlineStr">
+        <is>
+          <t>Андижанская</t>
+        </is>
+      </c>
+      <c r="C23" s="40" t="n">
+        <v>4967742</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="37" t="inlineStr">
+        <is>
+          <t>ИТОГО по сети</t>
+        </is>
+      </c>
+      <c r="B24" s="38" t="inlineStr"/>
+      <c r="C24" s="41">
+        <f>SUM(C6:C23)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
sync: +3 дня (09-11.06.2026); неделя 08.06-14.06 дни 1->3 (неполная)
</commit_message>
<xml_diff>
--- a/Эталон_ПВЗ.xlsx
+++ b/Эталон_ПВЗ.xlsx
@@ -2015,7 +2015,7 @@
         <v>7</v>
       </c>
       <c r="G5" s="34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -2042,7 +2042,7 @@
         <v>53</v>
       </c>
       <c r="G6" s="36" t="n">
-        <v>88</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7">
@@ -2069,7 +2069,7 @@
         <v>51.43</v>
       </c>
       <c r="G7" s="36" t="n">
-        <v>70</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8">
@@ -2096,142 +2096,142 @@
         <v>35.57</v>
       </c>
       <c r="G8" s="36" t="n">
-        <v>37</v>
+        <v>42.33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>FRТАШ-294</t>
+          <t>FRТАШ-289</t>
         </is>
       </c>
       <c r="B9" s="35" t="inlineStr">
         <is>
-          <t>Шастри</t>
+          <t>Афросиаб</t>
         </is>
       </c>
       <c r="C9" s="36" t="n">
-        <v>18.8</v>
+        <v>5.5</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>26.57</v>
+        <v>17.86</v>
       </c>
       <c r="E9" s="36" t="n">
-        <v>28.29</v>
+        <v>20.86</v>
       </c>
       <c r="F9" s="36" t="n">
-        <v>28.71</v>
+        <v>24.86</v>
       </c>
       <c r="G9" s="36" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>FRТАШ-293</t>
+          <t>FRТАШ-294</t>
         </is>
       </c>
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>Кургантепа</t>
+          <t>Шастри</t>
         </is>
       </c>
       <c r="C10" s="36" t="n">
-        <v>8</v>
+        <v>18.8</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>13</v>
+        <v>26.57</v>
       </c>
       <c r="E10" s="36" t="n">
-        <v>17.71</v>
+        <v>28.29</v>
       </c>
       <c r="F10" s="36" t="n">
-        <v>26.57</v>
+        <v>28.71</v>
       </c>
       <c r="G10" s="36" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>FRТАШ-289</t>
+          <t>FRТАШ-293</t>
         </is>
       </c>
       <c r="B11" s="35" t="inlineStr">
         <is>
-          <t>Афросиаб</t>
+          <t>Кургантепа</t>
         </is>
       </c>
       <c r="C11" s="36" t="n">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>17.86</v>
+        <v>13</v>
       </c>
       <c r="E11" s="36" t="n">
-        <v>20.86</v>
+        <v>17.71</v>
       </c>
       <c r="F11" s="36" t="n">
-        <v>24.86</v>
+        <v>26.57</v>
       </c>
       <c r="G11" s="36" t="n">
-        <v>26</v>
+        <v>27.67</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="35" t="inlineStr">
         <is>
-          <t>FRАЛМ-10</t>
+          <t>FRАЛМ-9</t>
         </is>
       </c>
       <c r="B12" s="35" t="inlineStr">
         <is>
-          <t>Алмалык Мустакилик</t>
+          <t>Алмалык Амир Т</t>
         </is>
       </c>
       <c r="C12" s="36" t="n">
-        <v>7.2</v>
+        <v>13.4</v>
       </c>
       <c r="D12" s="36" t="n">
-        <v>8.140000000000001</v>
+        <v>16.57</v>
       </c>
       <c r="E12" s="36" t="n">
-        <v>9.140000000000001</v>
+        <v>20.86</v>
       </c>
       <c r="F12" s="36" t="n">
-        <v>14.14</v>
+        <v>17.14</v>
       </c>
       <c r="G12" s="36" t="n">
-        <v>22</v>
+        <v>21.33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="35" t="inlineStr">
         <is>
-          <t>FRГАЗ-4</t>
+          <t>FRАЛМ-10</t>
         </is>
       </c>
       <c r="B13" s="35" t="inlineStr">
         <is>
-          <t>Газалкент</t>
+          <t>Алмалык Мустакилик</t>
         </is>
       </c>
       <c r="C13" s="36" t="n">
-        <v>9.6</v>
+        <v>7.2</v>
       </c>
       <c r="D13" s="36" t="n">
-        <v>13.29</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="E13" s="36" t="n">
-        <v>14.57</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="F13" s="36" t="n">
-        <v>16.71</v>
+        <v>14.14</v>
       </c>
       <c r="G13" s="36" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
@@ -2258,7 +2258,7 @@
         <v>17.57</v>
       </c>
       <c r="G14" s="36" t="n">
-        <v>19</v>
+        <v>19.67</v>
       </c>
     </row>
     <row r="15">
@@ -2285,34 +2285,34 @@
         <v>13.43</v>
       </c>
       <c r="G15" s="36" t="n">
-        <v>18</v>
+        <v>18.33</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="35" t="inlineStr">
         <is>
-          <t>FRАЛМ-9</t>
+          <t>FRБХР-30</t>
         </is>
       </c>
       <c r="B16" s="35" t="inlineStr">
         <is>
-          <t>Алмалык Амир Т</t>
+          <t>Бухара</t>
         </is>
       </c>
       <c r="C16" s="36" t="n">
-        <v>13.4</v>
+        <v>13.8</v>
       </c>
       <c r="D16" s="36" t="n">
-        <v>16.57</v>
+        <v>21.71</v>
       </c>
       <c r="E16" s="36" t="n">
-        <v>20.86</v>
+        <v>15.43</v>
       </c>
       <c r="F16" s="36" t="n">
-        <v>17.14</v>
+        <v>17</v>
       </c>
       <c r="G16" s="36" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17">
@@ -2339,88 +2339,88 @@
         <v>14.86</v>
       </c>
       <c r="G17" s="36" t="n">
-        <v>16</v>
+        <v>16.67</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="35" t="inlineStr">
         <is>
-          <t>FRБХР-30</t>
+          <t>FRГАЗ-4</t>
         </is>
       </c>
       <c r="B18" s="35" t="inlineStr">
         <is>
-          <t>Бухара</t>
+          <t>Газалкент</t>
         </is>
       </c>
       <c r="C18" s="36" t="n">
-        <v>13.8</v>
+        <v>9.6</v>
       </c>
       <c r="D18" s="36" t="n">
-        <v>21.71</v>
+        <v>13.29</v>
       </c>
       <c r="E18" s="36" t="n">
-        <v>15.43</v>
+        <v>14.57</v>
       </c>
       <c r="F18" s="36" t="n">
-        <v>17</v>
+        <v>16.71</v>
       </c>
       <c r="G18" s="36" t="n">
-        <v>14</v>
+        <v>16.67</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="35" t="inlineStr">
         <is>
-          <t>FRСМК-52</t>
+          <t>FRСМК-53</t>
         </is>
       </c>
       <c r="B19" s="35" t="inlineStr">
         <is>
-          <t>Рудаки</t>
+          <t>Андижанская</t>
         </is>
       </c>
       <c r="C19" s="36" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="D19" s="36" t="n">
-        <v>10.43</v>
+        <v>0.25</v>
       </c>
       <c r="E19" s="36" t="n">
-        <v>11.14</v>
+        <v>2.86</v>
       </c>
       <c r="F19" s="36" t="n">
-        <v>13.43</v>
+        <v>8.43</v>
       </c>
       <c r="G19" s="36" t="n">
-        <v>14</v>
+        <v>16.33</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="35" t="inlineStr">
         <is>
-          <t>FRСМК-53</t>
+          <t>FRСМК-52</t>
         </is>
       </c>
       <c r="B20" s="35" t="inlineStr">
         <is>
-          <t>Андижанская</t>
+          <t>Рудаки</t>
         </is>
       </c>
       <c r="C20" s="36" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D20" s="36" t="n">
-        <v>0.25</v>
+        <v>10.43</v>
       </c>
       <c r="E20" s="36" t="n">
-        <v>2.86</v>
+        <v>11.14</v>
       </c>
       <c r="F20" s="36" t="n">
-        <v>8.43</v>
+        <v>13.43</v>
       </c>
       <c r="G20" s="36" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21">
@@ -2447,7 +2447,7 @@
         <v>9.289999999999999</v>
       </c>
       <c r="G21" s="36" t="n">
-        <v>10</v>
+        <v>8.67</v>
       </c>
     </row>
     <row r="22">
@@ -2474,7 +2474,7 @@
         <v>5.86</v>
       </c>
       <c r="G22" s="36" t="n">
-        <v>5</v>
+        <v>5.67</v>
       </c>
     </row>
     <row r="23">
@@ -2501,7 +2501,7 @@
         <v>7.86</v>
       </c>
       <c r="G23" s="36" t="n">
-        <v>2</v>
+        <v>5.33</v>
       </c>
     </row>
     <row r="24">
@@ -2653,7 +2653,7 @@
         <v>7</v>
       </c>
       <c r="G5" s="34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -2680,7 +2680,7 @@
         <v>64308195</v>
       </c>
       <c r="G6" s="40" t="n">
-        <v>12733834</v>
+        <v>29173014</v>
       </c>
     </row>
     <row r="7">
@@ -2707,7 +2707,7 @@
         <v>52194797</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>11870686</v>
+        <v>31189340</v>
       </c>
     </row>
     <row r="8">
@@ -2734,142 +2734,142 @@
         <v>48937774</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>8996930</v>
+        <v>25021030</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>FRТАШ-294</t>
+          <t>FRТАШ-289</t>
         </is>
       </c>
       <c r="B9" s="35" t="inlineStr">
         <is>
-          <t>Шастри</t>
+          <t>Афросиаб</t>
         </is>
       </c>
       <c r="C9" s="40" t="n">
-        <v>11787061</v>
+        <v>3579870</v>
       </c>
       <c r="D9" s="40" t="n">
-        <v>33489630</v>
+        <v>26016508</v>
       </c>
       <c r="E9" s="40" t="n">
-        <v>34406847</v>
+        <v>28967720</v>
       </c>
       <c r="F9" s="40" t="n">
-        <v>37161831</v>
+        <v>37959389</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>4538440</v>
+        <v>20167263</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>FRТАШ-293</t>
+          <t>FRТАШ-294</t>
         </is>
       </c>
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>Кургантепа</t>
+          <t>Шастри</t>
         </is>
       </c>
       <c r="C10" s="40" t="n">
-        <v>9063650</v>
+        <v>11787061</v>
       </c>
       <c r="D10" s="40" t="n">
-        <v>19435779</v>
+        <v>33489630</v>
       </c>
       <c r="E10" s="40" t="n">
-        <v>20382320</v>
+        <v>34406847</v>
       </c>
       <c r="F10" s="40" t="n">
-        <v>23759937</v>
+        <v>37161831</v>
       </c>
       <c r="G10" s="40" t="n">
-        <v>5677190</v>
+        <v>11579824</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>FRТАШ-289</t>
+          <t>FRТАШ-293</t>
         </is>
       </c>
       <c r="B11" s="35" t="inlineStr">
         <is>
-          <t>Афросиаб</t>
+          <t>Кургантепа</t>
         </is>
       </c>
       <c r="C11" s="40" t="n">
-        <v>3579870</v>
+        <v>9063650</v>
       </c>
       <c r="D11" s="40" t="n">
-        <v>26016508</v>
+        <v>19435779</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>28967720</v>
+        <v>20382320</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>37959389</v>
+        <v>23759937</v>
       </c>
       <c r="G11" s="40" t="n">
-        <v>5645596</v>
+        <v>16411118</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="35" t="inlineStr">
         <is>
-          <t>FRАЛМ-10</t>
+          <t>FRАЛМ-9</t>
         </is>
       </c>
       <c r="B12" s="35" t="inlineStr">
         <is>
-          <t>Алмалык Мустакилик</t>
+          <t>Алмалык Амир Т</t>
         </is>
       </c>
       <c r="C12" s="40" t="n">
-        <v>6011315</v>
+        <v>13421812</v>
       </c>
       <c r="D12" s="40" t="n">
-        <v>10213590</v>
+        <v>19296100</v>
       </c>
       <c r="E12" s="40" t="n">
-        <v>10032796</v>
+        <v>32898025</v>
       </c>
       <c r="F12" s="40" t="n">
-        <v>23828037</v>
+        <v>20322786</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>6409560</v>
+        <v>14234181</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="35" t="inlineStr">
         <is>
-          <t>FRГАЗ-4</t>
+          <t>FRАЛМ-10</t>
         </is>
       </c>
       <c r="B13" s="35" t="inlineStr">
         <is>
-          <t>Газалкент</t>
+          <t>Алмалык Мустакилик</t>
         </is>
       </c>
       <c r="C13" s="40" t="n">
-        <v>6139086</v>
+        <v>6011315</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>14744333</v>
+        <v>10213590</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>18390296</v>
+        <v>10032796</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>19525644</v>
+        <v>23828037</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>3737250</v>
+        <v>22340500</v>
       </c>
     </row>
     <row r="14">
@@ -2896,7 +2896,7 @@
         <v>20628257</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>1866491</v>
+        <v>7602741</v>
       </c>
     </row>
     <row r="15">
@@ -2923,34 +2923,34 @@
         <v>18213851</v>
       </c>
       <c r="G15" s="40" t="n">
-        <v>1807552</v>
+        <v>8786876</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="35" t="inlineStr">
         <is>
-          <t>FRАЛМ-9</t>
+          <t>FRБХР-30</t>
         </is>
       </c>
       <c r="B16" s="35" t="inlineStr">
         <is>
-          <t>Алмалык Амир Т</t>
+          <t>Бухара</t>
         </is>
       </c>
       <c r="C16" s="40" t="n">
-        <v>13421812</v>
+        <v>10462042</v>
       </c>
       <c r="D16" s="40" t="n">
-        <v>19296100</v>
+        <v>24242808</v>
       </c>
       <c r="E16" s="40" t="n">
-        <v>32898025</v>
+        <v>20176647</v>
       </c>
       <c r="F16" s="40" t="n">
-        <v>20322786</v>
+        <v>18937286</v>
       </c>
       <c r="G16" s="40" t="n">
-        <v>1421720</v>
+        <v>7992670</v>
       </c>
     </row>
     <row r="17">
@@ -2977,88 +2977,88 @@
         <v>18898662</v>
       </c>
       <c r="G17" s="40" t="n">
-        <v>2122384</v>
+        <v>6622614</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="35" t="inlineStr">
         <is>
-          <t>FRБХР-30</t>
+          <t>FRГАЗ-4</t>
         </is>
       </c>
       <c r="B18" s="35" t="inlineStr">
         <is>
-          <t>Бухара</t>
+          <t>Газалкент</t>
         </is>
       </c>
       <c r="C18" s="40" t="n">
-        <v>10462042</v>
+        <v>6139086</v>
       </c>
       <c r="D18" s="40" t="n">
-        <v>24242808</v>
+        <v>14744333</v>
       </c>
       <c r="E18" s="40" t="n">
-        <v>20176647</v>
+        <v>18390296</v>
       </c>
       <c r="F18" s="40" t="n">
-        <v>18937286</v>
+        <v>19525644</v>
       </c>
       <c r="G18" s="40" t="n">
-        <v>2589400</v>
+        <v>7061536</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="35" t="inlineStr">
         <is>
-          <t>FRСМК-52</t>
+          <t>FRСМК-53</t>
         </is>
       </c>
       <c r="B19" s="35" t="inlineStr">
         <is>
-          <t>Рудаки</t>
+          <t>Андижанская</t>
         </is>
       </c>
       <c r="C19" s="40" t="n">
-        <v>6460094</v>
+        <v>0</v>
       </c>
       <c r="D19" s="40" t="n">
-        <v>14908071</v>
+        <v>363900</v>
       </c>
       <c r="E19" s="40" t="n">
-        <v>20904887</v>
+        <v>3477490</v>
       </c>
       <c r="F19" s="40" t="n">
-        <v>14174417</v>
+        <v>6698688</v>
       </c>
       <c r="G19" s="40" t="n">
-        <v>2274090</v>
+        <v>6132968</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="35" t="inlineStr">
         <is>
-          <t>FRСМК-53</t>
+          <t>FRСМК-52</t>
         </is>
       </c>
       <c r="B20" s="35" t="inlineStr">
         <is>
-          <t>Андижанская</t>
+          <t>Рудаки</t>
         </is>
       </c>
       <c r="C20" s="40" t="n">
-        <v>0</v>
+        <v>6460094</v>
       </c>
       <c r="D20" s="40" t="n">
-        <v>363900</v>
+        <v>14908071</v>
       </c>
       <c r="E20" s="40" t="n">
-        <v>3477490</v>
+        <v>20904887</v>
       </c>
       <c r="F20" s="40" t="n">
-        <v>6698688</v>
+        <v>14174417</v>
       </c>
       <c r="G20" s="40" t="n">
-        <v>2340920</v>
+        <v>5800193</v>
       </c>
     </row>
     <row r="21">
@@ -3085,7 +3085,7 @@
         <v>18439963</v>
       </c>
       <c r="G21" s="40" t="n">
-        <v>491910</v>
+        <v>3475570</v>
       </c>
     </row>
     <row r="22">
@@ -3112,7 +3112,7 @@
         <v>4464440</v>
       </c>
       <c r="G22" s="40" t="n">
-        <v>4980680</v>
+        <v>7713840</v>
       </c>
     </row>
     <row r="23">
@@ -3139,7 +3139,7 @@
         <v>7337990</v>
       </c>
       <c r="G23" s="40" t="n">
-        <v>207910</v>
+        <v>2995030</v>
       </c>
     </row>
     <row r="24">
@@ -3291,7 +3291,7 @@
         <v>7</v>
       </c>
       <c r="G5" s="34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -3318,7 +3318,7 @@
         <v>7</v>
       </c>
       <c r="G6" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -3345,7 +3345,7 @@
         <v>7</v>
       </c>
       <c r="G7" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -3372,22 +3372,22 @@
         <v>7</v>
       </c>
       <c r="G8" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="35" t="inlineStr">
         <is>
-          <t>FRТАШ-294</t>
+          <t>FRТАШ-289</t>
         </is>
       </c>
       <c r="B9" s="35" t="inlineStr">
         <is>
-          <t>Шастри</t>
+          <t>Афросиаб</t>
         </is>
       </c>
       <c r="C9" s="42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" s="42" t="n">
         <v>7</v>
@@ -3399,18 +3399,18 @@
         <v>7</v>
       </c>
       <c r="G9" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="35" t="inlineStr">
         <is>
-          <t>FRТАШ-293</t>
+          <t>FRТАШ-294</t>
         </is>
       </c>
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>Кургантепа</t>
+          <t>Шастри</t>
         </is>
       </c>
       <c r="C10" s="42" t="n">
@@ -3426,22 +3426,22 @@
         <v>7</v>
       </c>
       <c r="G10" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="35" t="inlineStr">
         <is>
-          <t>FRТАШ-289</t>
+          <t>FRТАШ-293</t>
         </is>
       </c>
       <c r="B11" s="35" t="inlineStr">
         <is>
-          <t>Афросиаб</t>
+          <t>Кургантепа</t>
         </is>
       </c>
       <c r="C11" s="42" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D11" s="42" t="n">
         <v>7</v>
@@ -3453,18 +3453,18 @@
         <v>7</v>
       </c>
       <c r="G11" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="35" t="inlineStr">
         <is>
-          <t>FRАЛМ-10</t>
+          <t>FRАЛМ-9</t>
         </is>
       </c>
       <c r="B12" s="35" t="inlineStr">
         <is>
-          <t>Алмалык Мустакилик</t>
+          <t>Алмалык Амир Т</t>
         </is>
       </c>
       <c r="C12" s="42" t="n">
@@ -3480,18 +3480,18 @@
         <v>7</v>
       </c>
       <c r="G12" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="35" t="inlineStr">
         <is>
-          <t>FRГАЗ-4</t>
+          <t>FRАЛМ-10</t>
         </is>
       </c>
       <c r="B13" s="35" t="inlineStr">
         <is>
-          <t>Газалкент</t>
+          <t>Алмалык Мустакилик</t>
         </is>
       </c>
       <c r="C13" s="42" t="n">
@@ -3507,7 +3507,7 @@
         <v>7</v>
       </c>
       <c r="G13" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -3534,7 +3534,7 @@
         <v>7</v>
       </c>
       <c r="G14" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -3561,18 +3561,18 @@
         <v>7</v>
       </c>
       <c r="G15" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="35" t="inlineStr">
         <is>
-          <t>FRАЛМ-9</t>
+          <t>FRБХР-30</t>
         </is>
       </c>
       <c r="B16" s="35" t="inlineStr">
         <is>
-          <t>Алмалык Амир Т</t>
+          <t>Бухара</t>
         </is>
       </c>
       <c r="C16" s="42" t="n">
@@ -3588,7 +3588,7 @@
         <v>7</v>
       </c>
       <c r="G16" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -3615,18 +3615,18 @@
         <v>7</v>
       </c>
       <c r="G17" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="35" t="inlineStr">
         <is>
-          <t>FRБХР-30</t>
+          <t>FRГАЗ-4</t>
         </is>
       </c>
       <c r="B18" s="35" t="inlineStr">
         <is>
-          <t>Бухара</t>
+          <t>Газалкент</t>
         </is>
       </c>
       <c r="C18" s="42" t="n">
@@ -3642,25 +3642,25 @@
         <v>7</v>
       </c>
       <c r="G18" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="35" t="inlineStr">
         <is>
-          <t>FRСМК-52</t>
+          <t>FRСМК-53</t>
         </is>
       </c>
       <c r="B19" s="35" t="inlineStr">
         <is>
-          <t>Рудаки</t>
+          <t>Андижанская</t>
         </is>
       </c>
       <c r="C19" s="42" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D19" s="42" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E19" s="42" t="n">
         <v>7</v>
@@ -3669,25 +3669,25 @@
         <v>7</v>
       </c>
       <c r="G19" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="35" t="inlineStr">
         <is>
-          <t>FRСМК-53</t>
+          <t>FRСМК-52</t>
         </is>
       </c>
       <c r="B20" s="35" t="inlineStr">
         <is>
-          <t>Андижанская</t>
+          <t>Рудаки</t>
         </is>
       </c>
       <c r="C20" s="42" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D20" s="42" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E20" s="42" t="n">
         <v>7</v>
@@ -3696,7 +3696,7 @@
         <v>7</v>
       </c>
       <c r="G20" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -3723,7 +3723,7 @@
         <v>7</v>
       </c>
       <c r="G21" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -3750,7 +3750,7 @@
         <v>7</v>
       </c>
       <c r="G22" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -3777,7 +3777,7 @@
         <v>7</v>
       </c>
       <c r="G23" s="42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">

</xml_diff>